<commit_message>
Modify UI for more  user-friendly interface
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_31055733_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_31055733_table1_v1.xlsx
@@ -928,7 +928,7 @@
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>MIR548AB</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>MIR548AB</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>MIR548AB</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>NRSN1</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>GRIN2B</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>SLC2A13</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>SMARCE1</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>RNF152</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>MIR4432</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>LINC01060</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>LINGO2</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>MIR7154,CHST1</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>MIR7154,CHST1</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>MIR7154,CHST1</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>CATSPERB</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>ATP5J</t>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>